<commit_message>
feat: import operator assign, batch filters, export clean and uppercase
导入可选操作员列自动分配；管理端批次筛选；导出清洗与正式库英文字母大写；构建前端 dist。

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/需求相关/分类平台表头.xlsx
+++ b/需求相关/分类平台表头.xlsx
@@ -1,264 +1,184 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375" tabRatio="721"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="12375" tabRatio="721" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="14" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t>序号</t>
-  </si>
-  <si>
-    <t>宝贝ID</t>
-  </si>
-  <si>
-    <t>宝贝主图</t>
-  </si>
-  <si>
-    <t>宝贝名称</t>
-  </si>
-  <si>
-    <t>品牌</t>
-  </si>
-  <si>
-    <t>是否经营</t>
-  </si>
-  <si>
-    <t>大类</t>
-  </si>
-  <si>
-    <t>区隔</t>
-  </si>
-  <si>
-    <t>类别</t>
-  </si>
-  <si>
-    <t>主材质</t>
-  </si>
-  <si>
-    <t>辅材质</t>
-  </si>
-  <si>
-    <t>包装方式</t>
-  </si>
-  <si>
-    <t>尺寸</t>
-  </si>
-  <si>
-    <t>卷数</t>
-  </si>
-  <si>
-    <t>总入数</t>
-  </si>
-  <si>
-    <t>产品属性</t>
-  </si>
-  <si>
-    <t>宝贝文描图</t>
-  </si>
-  <si>
-    <t>宝贝链接</t>
-  </si>
-  <si>
-    <t>数据平台</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="21">
     <font>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -558,164 +478,165 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -769,16 +690,7 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="000000FF"/>
-    </mruColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -1067,78 +979,123 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="3" max="3" width="29" customWidth="1"/>
-    <col min="4" max="4" width="11.5583333333333" customWidth="1"/>
-    <col min="17" max="17" width="12.125" customWidth="1"/>
-    <col min="18" max="18" width="10.25" customWidth="1"/>
+    <col width="29" customWidth="1" style="3" min="3" max="3"/>
+    <col width="11.5583333333333" customWidth="1" style="3" min="4" max="4"/>
+    <col width="12.125" customWidth="1" style="3" min="17" max="17"/>
+    <col width="10.25" customWidth="1" style="3" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>18</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>宝贝ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>宝贝主图</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>宝贝名称</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>品牌</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>是否经营</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>大类</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>区隔</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>类别</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>主材质</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>辅材质</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>包装方式</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>尺寸</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>卷数</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>总入数</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>产品属性</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>宝贝文描图</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>宝贝链接</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>数据平台</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>操作员</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>